<commit_message>
feat(reminders): add Gmail Apps Script reminder flow and backend reminder candidates endpoint
</commit_message>
<xml_diff>
--- a/server/data/feedback_store.xlsx
+++ b/server/data/feedback_store.xlsx
@@ -12,6 +12,7 @@
     <sheet name="summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="feedback" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ingestion_queue" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1804,9 +1805,6 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>2026-03-01T09:45:02Z</t>
@@ -1835,17 +1833,12 @@
       <c r="N5" t="n">
         <v>4.5</v>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
         <v>3.5</v>
       </c>
       <c r="R5" t="n">
         <v>3.8</v>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
         <v>3.5</v>
       </c>
@@ -1975,19 +1968,70 @@
       <c r="G2" t="n">
         <v>4.5</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>3.5</v>
       </c>
       <c r="K2" t="n">
         <v>3.8</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>3.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attempt_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>next_retry_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>last_error</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>payload_json</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>